<commit_message>
se agrega pantalla medio de pago
</commit_message>
<xml_diff>
--- a/documentos/Funcionalidades.xlsx
+++ b/documentos/Funcionalidades.xlsx
@@ -5,19 +5,20 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Documentos\proyecto_minimarket\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\mis-proyectos\gestion-minimarket\documentos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42302B17-A851-4E7E-ADB7-E058794C003B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD1664A3-E307-41AB-A89E-2967AC0EC78F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Inventario" sheetId="1" r:id="rId1"/>
     <sheet name="Tablas" sheetId="2" r:id="rId2"/>
-    <sheet name="Requerimientos" sheetId="3" r:id="rId3"/>
-    <sheet name="Bd_usuarios" sheetId="4" r:id="rId4"/>
-    <sheet name="Nuevas funcionalidades" sheetId="5" r:id="rId5"/>
+    <sheet name="To Do" sheetId="6" r:id="rId3"/>
+    <sheet name="Requerimientos" sheetId="3" r:id="rId4"/>
+    <sheet name="Bd_usuarios" sheetId="4" r:id="rId5"/>
+    <sheet name="Nuevas funcionalidades" sheetId="5" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -204,7 +205,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="212" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="225" uniqueCount="118">
   <si>
     <t>Registro de producto</t>
   </si>
@@ -552,6 +553,24 @@
   </si>
   <si>
     <t>idposshift</t>
+  </si>
+  <si>
+    <t>PaymentMethods</t>
+  </si>
+  <si>
+    <t>payments</t>
+  </si>
+  <si>
+    <t>id payment</t>
+  </si>
+  <si>
+    <t>monto</t>
+  </si>
+  <si>
+    <t>Al registrar el producto no se muestra las categorias, se creo golosinas y no se muestra</t>
+  </si>
+  <si>
+    <t>Al registrar el producto, verificar que se registre en la tabla de inventario o kardex</t>
   </si>
 </sst>
 </file>
@@ -766,8 +785,10 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1184,7 +1205,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C46C0296-A8C3-417B-A850-4DA7BD8456BD}">
-  <dimension ref="A2:Q40"/>
+  <dimension ref="A2:Q46"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="2.81640625" bestFit="1" customWidth="1"/>
@@ -1695,9 +1716,7 @@
         <v>66</v>
       </c>
       <c r="P23" s="8"/>
-      <c r="Q23" s="8" t="s">
-        <v>44</v>
-      </c>
+      <c r="Q23" s="8"/>
     </row>
     <row r="24" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A24" s="8"/>
@@ -1725,7 +1744,7 @@
       <c r="J25" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="K25" s="19" t="s">
+      <c r="K25" s="8" t="s">
         <v>62</v>
       </c>
       <c r="M25" s="8"/>
@@ -1743,7 +1762,7 @@
       <c r="J26" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="K26" s="19" t="s">
+      <c r="K26" s="8" t="s">
         <v>102</v>
       </c>
       <c r="M26" s="8"/>
@@ -1776,11 +1795,9 @@
       <c r="K28" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="M28" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="N28" s="17" t="s">
-        <v>62</v>
+      <c r="M28" s="8"/>
+      <c r="N28" s="20" t="s">
+        <v>113</v>
       </c>
     </row>
     <row r="29" spans="1:17" x14ac:dyDescent="0.35">
@@ -1788,19 +1805,15 @@
       <c r="B29" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="M29" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="N29" s="17" t="s">
-        <v>102</v>
+      <c r="M29" s="8"/>
+      <c r="N29" s="9" t="s">
+        <v>114</v>
       </c>
     </row>
     <row r="30" spans="1:17" x14ac:dyDescent="0.35">
-      <c r="M30" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="N30" s="17" t="s">
-        <v>111</v>
+      <c r="M30" s="8"/>
+      <c r="N30" s="9" t="s">
+        <v>115</v>
       </c>
     </row>
     <row r="31" spans="1:17" x14ac:dyDescent="0.35">
@@ -1809,9 +1822,7 @@
         <v>104</v>
       </c>
       <c r="M31" s="8"/>
-      <c r="N31" s="8" t="s">
-        <v>12</v>
-      </c>
+      <c r="N31" s="12"/>
     </row>
     <row r="32" spans="1:17" x14ac:dyDescent="0.35">
       <c r="J32" s="8" t="s">
@@ -1820,42 +1831,64 @@
       <c r="K32" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="M32" s="8"/>
-      <c r="N32" s="8" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="33" spans="10:11" x14ac:dyDescent="0.35">
+      <c r="M32" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="N32" s="17" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="33" spans="10:14" x14ac:dyDescent="0.35">
       <c r="J33" s="8"/>
       <c r="K33" s="8" t="s">
         <v>106</v>
       </c>
-    </row>
-    <row r="34" spans="10:11" x14ac:dyDescent="0.35">
+      <c r="M33" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="N33" s="17" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="34" spans="10:14" x14ac:dyDescent="0.35">
       <c r="J34" s="8"/>
       <c r="K34" s="8" t="s">
         <v>107</v>
       </c>
-    </row>
-    <row r="35" spans="10:11" x14ac:dyDescent="0.35">
+      <c r="M34" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="N34" s="17" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="35" spans="10:14" x14ac:dyDescent="0.35">
       <c r="J35" s="8"/>
       <c r="K35" s="8" t="s">
         <v>108</v>
       </c>
-    </row>
-    <row r="36" spans="10:11" x14ac:dyDescent="0.35">
+      <c r="M35" s="8"/>
+      <c r="N35" s="8" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="36" spans="10:14" x14ac:dyDescent="0.35">
       <c r="J36" s="8"/>
       <c r="K36" s="8" t="s">
         <v>109</v>
       </c>
-    </row>
-    <row r="37" spans="10:11" x14ac:dyDescent="0.35">
+      <c r="M36" s="8"/>
+      <c r="N36" s="8" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="37" spans="10:14" x14ac:dyDescent="0.35">
       <c r="J37" s="8"/>
       <c r="K37" s="8" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="38" spans="10:11" x14ac:dyDescent="0.35">
+    <row r="38" spans="10:14" x14ac:dyDescent="0.35">
       <c r="J38" s="8" t="s">
         <v>16</v>
       </c>
@@ -1863,20 +1896,66 @@
         <v>105</v>
       </c>
     </row>
-    <row r="39" spans="10:11" x14ac:dyDescent="0.35">
+    <row r="39" spans="10:14" x14ac:dyDescent="0.35">
       <c r="J39" t="s">
         <v>16</v>
       </c>
-      <c r="K39" s="20" t="s">
+      <c r="K39" s="19" t="s">
         <v>102</v>
       </c>
-    </row>
-    <row r="40" spans="10:11" x14ac:dyDescent="0.35">
+      <c r="M39" s="8"/>
+      <c r="N39" s="8" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="40" spans="10:14" x14ac:dyDescent="0.35">
       <c r="J40" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="K40" s="19" t="s">
+      <c r="K40" s="8" t="s">
         <v>62</v>
+      </c>
+      <c r="M40" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="N40" s="8" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="41" spans="10:14" x14ac:dyDescent="0.35">
+      <c r="M41" s="8"/>
+      <c r="N41" s="8" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="42" spans="10:14" x14ac:dyDescent="0.35">
+      <c r="M42" s="8"/>
+      <c r="N42" s="8" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="43" spans="10:14" x14ac:dyDescent="0.35">
+      <c r="M43" s="8"/>
+      <c r="N43" s="8" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="44" spans="10:14" x14ac:dyDescent="0.35">
+      <c r="M44" s="8"/>
+      <c r="N44" s="8" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="45" spans="10:14" x14ac:dyDescent="0.35">
+      <c r="M45" s="8"/>
+      <c r="N45" s="8" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="46" spans="10:14" x14ac:dyDescent="0.35">
+      <c r="M46" s="8"/>
+      <c r="N46" s="8" t="s">
+        <v>13</v>
       </c>
     </row>
   </sheetData>
@@ -1886,6 +1965,26 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D3A6A09D-0BA8-407E-BCA0-8B0EE64B8D07}">
+  <dimension ref="A2:A3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>117</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4386CA15-4375-4961-8873-24B5219F2ECC}">
   <dimension ref="A3:A19"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -1962,7 +2061,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{83BAD629-A18D-4736-8D2D-A5B06CBAF5F0}">
   <dimension ref="B2:F10"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -2051,7 +2150,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0724688A-8298-4485-ACBD-A429C8451820}">
   <dimension ref="A3:A14"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>

</xml_diff>

<commit_message>
ajuste de ventas e impresion y cierre de caja
</commit_message>
<xml_diff>
--- a/documentos/Funcionalidades.xlsx
+++ b/documentos/Funcionalidades.xlsx
@@ -1,24 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27830"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28925"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\mis-proyectos\gestion-minimarket\documentos\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\workspace\personal\gestion-minimarket\documentos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD1664A3-E307-41AB-A89E-2967AC0EC78F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EFD820DC-22AC-48D4-8761-34A49BB9DB30}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Inventario" sheetId="1" r:id="rId1"/>
     <sheet name="Tablas" sheetId="2" r:id="rId2"/>
     <sheet name="To Do" sheetId="6" r:id="rId3"/>
-    <sheet name="Requerimientos" sheetId="3" r:id="rId4"/>
-    <sheet name="Bd_usuarios" sheetId="4" r:id="rId5"/>
-    <sheet name="Nuevas funcionalidades" sheetId="5" r:id="rId6"/>
+    <sheet name="funcionalidades" sheetId="8" r:id="rId4"/>
+    <sheet name="Hoja1" sheetId="7" r:id="rId5"/>
+    <sheet name="Requerimientos" sheetId="3" r:id="rId6"/>
+    <sheet name="Bd_usuarios" sheetId="4" r:id="rId7"/>
+    <sheet name="Nuevas funcionalidades" sheetId="5" r:id="rId8"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -205,7 +207,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="225" uniqueCount="118">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="287" uniqueCount="166">
   <si>
     <t>Registro de producto</t>
   </si>
@@ -567,10 +569,154 @@
     <t>monto</t>
   </si>
   <si>
-    <t>Al registrar el producto no se muestra las categorias, se creo golosinas y no se muestra</t>
-  </si>
-  <si>
-    <t>Al registrar el producto, verificar que se registre en la tabla de inventario o kardex</t>
+    <t>Mejora para manejar el tipo de documento y serie.</t>
+  </si>
+  <si>
+    <t>Mejora tecnica, cuando se intente acceder directamente a una url no se puede porque no está autorizado, entonces debería enviar a la pantalla de inicio de sesion</t>
+  </si>
+  <si>
+    <t>Controla los accesos: solo usuarios autorizados pueden hacer ajustes de inventario, anular ventas o modificar pagos.</t>
+  </si>
+  <si>
+    <t>Mejora al cerrar la caja, que pasa si en el dia necesito retirar dinero de caja por algún motivo: compra de articulos, pago a proveedor.</t>
+  </si>
+  <si>
+    <t>Mejorar al pagar, que el monto total aparesca establecido la primera vez que se va pagar y que este todo seleccionado.</t>
+  </si>
+  <si>
+    <t>Mejora despues de cerrar la caja, se necesita una pantalla para consultar los datos del cierre de caja.</t>
+  </si>
+  <si>
+    <t>Mejora despues de pagar o cerrar caja, se necesita una pantalla para consultar las ventas.</t>
+  </si>
+  <si>
+    <t>venta</t>
+  </si>
+  <si>
+    <t>vuelto</t>
+  </si>
+  <si>
+    <t>pagos</t>
+  </si>
+  <si>
+    <t>efectivo</t>
+  </si>
+  <si>
+    <t>total ventas</t>
+  </si>
+  <si>
+    <t>total ingreso efectivo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">total vuelto en efectivo </t>
+  </si>
+  <si>
+    <t>yape</t>
+  </si>
+  <si>
+    <t>total ingreso yape</t>
+  </si>
+  <si>
+    <t>total vuelto en efectivo</t>
+  </si>
+  <si>
+    <t>total vuelto efectivo</t>
+  </si>
+  <si>
+    <t>Cambiar el boton editar para que sea sensible en todos los mantenimientos.</t>
+  </si>
+  <si>
+    <t>Mantenimiento y registro de productos</t>
+  </si>
+  <si>
+    <t>El código no debe ser obligatorio para productos sin codigo</t>
+  </si>
+  <si>
+    <t>Al editar que se muestre stock pero desabilitado</t>
+  </si>
+  <si>
+    <t>Al guardar la edición falta que guarde el stock minimo en la tabla stock producto</t>
+  </si>
+  <si>
+    <t>El boton editar tiene que ser mas sensible</t>
+  </si>
+  <si>
+    <t>Estado</t>
+  </si>
+  <si>
+    <t>DONE</t>
+  </si>
+  <si>
+    <t>Crear registro con otra Medida de venta, Presentación y Categoria.</t>
+  </si>
+  <si>
+    <t>Categoria no se edita</t>
+  </si>
+  <si>
+    <t>La categoria debe leer de la tabla correcta</t>
+  </si>
+  <si>
+    <t>Agregar el campo costo y que no sea obligatorio</t>
+  </si>
+  <si>
+    <t>Mantenimiento de Inventario</t>
+  </si>
+  <si>
+    <t>Ventas</t>
+  </si>
+  <si>
+    <t>Compras</t>
+  </si>
+  <si>
+    <t>Ingreso de productos al stock</t>
+  </si>
+  <si>
+    <t>Salida por merma</t>
+  </si>
+  <si>
+    <t>Salida por ajuste</t>
+  </si>
+  <si>
+    <t>Ingreso por el tema de compras</t>
+  </si>
+  <si>
+    <t>Ingreso por devolucion</t>
+  </si>
+  <si>
+    <t>En la compra tener en cuenta el costo y actualizarlo, tambien precio</t>
+  </si>
+  <si>
+    <t>Actualizar stock y se podría actualizar el precio/costo</t>
+  </si>
+  <si>
+    <t>Actualizar stock</t>
+  </si>
+  <si>
+    <t>Registrar producto rapido</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Maestro de unidad de venta, KL, UN, </t>
+  </si>
+  <si>
+    <t>Maestro de motivo de movimiento o reason transaccion</t>
+  </si>
+  <si>
+    <t>CORREGIR LA PANTALLA YA QUE SE MALOGRO POR TODO LAS MODIFICAINES QUE SE HIZO</t>
+  </si>
+  <si>
+    <t>AL REGISTRAR INGRESO ACTUALIZAR EN STOCKPRODUCTO, IGUAL EN SALIDA</t>
+  </si>
+  <si>
+    <t>Colocar en todos los botones para eliminar el puntero de manito y si es posible un poco mas grande</t>
+  </si>
+  <si>
+    <t>Implementar mejora para manejar el stock por tienda.</t>
+  </si>
+  <si>
+    <t>Implementar mejora para manejar el stock y el calculo de las utilidades por el inventario correcto.</t>
+  </si>
+  <si>
+    <t>Salida de prodcutos del stock</t>
   </si>
 </sst>
 </file>
@@ -753,7 +899,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
@@ -787,6 +933,9 @@
     <xf numFmtId="0" fontId="1" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -1966,17 +2115,62 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D3A6A09D-0BA8-407E-BCA0-8B0EE64B8D07}">
-  <dimension ref="A2:A3"/>
+  <dimension ref="A5:A22"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
         <v>117</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
+        <v>162</v>
       </c>
     </row>
   </sheetData>
@@ -1985,6 +2179,325 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7E042AC5-00C0-43A1-B25B-F04151E928AE}">
+  <dimension ref="A2:B38"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="71" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B2" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A4" s="10" t="s">
+        <v>136</v>
+      </c>
+      <c r="B4" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A5" s="10" t="s">
+        <v>137</v>
+      </c>
+      <c r="B5" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A6" s="10" t="s">
+        <v>138</v>
+      </c>
+      <c r="B6" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A7" s="10" t="s">
+        <v>139</v>
+      </c>
+      <c r="B7" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A8" s="10" t="s">
+        <v>142</v>
+      </c>
+      <c r="B8" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A9" s="10" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A10" s="10" t="s">
+        <v>144</v>
+      </c>
+      <c r="B10" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A11" s="10" t="s">
+        <v>145</v>
+      </c>
+      <c r="B11" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A14" s="21" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A15" s="10" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A16" s="10" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A17" s="10" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A18" s="10" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A19" s="10" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A20" s="10" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A21" s="10" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A22" s="10" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A23" s="10" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A24" s="10" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A25" s="10"/>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A26" s="10"/>
+    </row>
+    <row r="27" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A27" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A28" s="10" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A29" s="10" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="32" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A32" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="37" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A37" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="38" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A38" t="s">
+        <v>159</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C5DE46E6-C6DE-458B-A6E4-B5EA637CF075}">
+  <dimension ref="B3:G22"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="6" max="6" width="20.36328125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B3" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="5" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B5" t="s">
+        <v>66</v>
+      </c>
+      <c r="C5">
+        <v>90</v>
+      </c>
+      <c r="F5" t="s">
+        <v>127</v>
+      </c>
+      <c r="G5">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="6" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B6" t="s">
+        <v>124</v>
+      </c>
+      <c r="C6">
+        <v>10</v>
+      </c>
+      <c r="F6" t="s">
+        <v>128</v>
+      </c>
+      <c r="G6">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="7" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B7" t="s">
+        <v>125</v>
+      </c>
+      <c r="F7" t="s">
+        <v>129</v>
+      </c>
+      <c r="G7">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="8" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B8" s="10" t="s">
+        <v>126</v>
+      </c>
+      <c r="C8">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="12" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B12" t="s">
+        <v>66</v>
+      </c>
+      <c r="C12">
+        <v>170</v>
+      </c>
+      <c r="F12" t="s">
+        <v>127</v>
+      </c>
+      <c r="G12">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="13" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B13" t="s">
+        <v>125</v>
+      </c>
+      <c r="F13" t="s">
+        <v>131</v>
+      </c>
+      <c r="G13">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="14" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B14" s="10" t="s">
+        <v>130</v>
+      </c>
+      <c r="C14">
+        <v>200</v>
+      </c>
+      <c r="F14" t="s">
+        <v>132</v>
+      </c>
+      <c r="G14">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="15" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B15" t="s">
+        <v>124</v>
+      </c>
+      <c r="C15">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="19" spans="6:7" x14ac:dyDescent="0.35">
+      <c r="F19" t="s">
+        <v>127</v>
+      </c>
+      <c r="G19">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="20" spans="6:7" x14ac:dyDescent="0.35">
+      <c r="F20" t="s">
+        <v>128</v>
+      </c>
+      <c r="G20">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="21" spans="6:7" x14ac:dyDescent="0.35">
+      <c r="F21" t="s">
+        <v>131</v>
+      </c>
+      <c r="G21">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="22" spans="6:7" x14ac:dyDescent="0.35">
+      <c r="F22" t="s">
+        <v>133</v>
+      </c>
+      <c r="G22">
+        <v>40</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4386CA15-4375-4961-8873-24B5219F2ECC}">
   <dimension ref="A3:A19"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -2061,7 +2574,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{83BAD629-A18D-4736-8D2D-A5B06CBAF5F0}">
   <dimension ref="B2:F10"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -2150,7 +2663,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0724688A-8298-4485-ACBD-A429C8451820}">
   <dimension ref="A3:A14"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>

</xml_diff>

<commit_message>
se mejora registro de producto y motivo de transaccion
</commit_message>
<xml_diff>
--- a/documentos/Funcionalidades.xlsx
+++ b/documentos/Funcionalidades.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\workspace\personal\gestion-minimarket\documentos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EFD820DC-22AC-48D4-8761-34A49BB9DB30}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC40F5E6-4ECB-475F-B5BE-D3A02FCABD46}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="807" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Inventario" sheetId="1" r:id="rId1"/>
@@ -207,7 +207,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="287" uniqueCount="166">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="297" uniqueCount="176">
   <si>
     <t>Registro de producto</t>
   </si>
@@ -717,6 +717,36 @@
   </si>
   <si>
     <t>Salida de prodcutos del stock</t>
+  </si>
+  <si>
+    <t>Mejoras rapidas</t>
+  </si>
+  <si>
+    <t>códigos de barra debe ser string</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Number (limitado)	✅ String (EAN-13)</t>
+  </si>
+  <si>
+    <t>stock no debe ser neagtivo en base de datos</t>
+  </si>
+  <si>
+    <t>trazabilidad de la venta en inventario</t>
+  </si>
+  <si>
+    <t>precios por tienda</t>
+  </si>
+  <si>
+    <t>Precio por tienda (solo global).</t>
+  </si>
+  <si>
+    <t>Reserva/consistencia de stock ante múltiples cajas.</t>
+  </si>
+  <si>
+    <t>Movimientos de inventario trazables (saleId / purchaseId).</t>
+  </si>
+  <si>
+    <t>promedio de costo y actualización automática.</t>
   </si>
 </sst>
 </file>
@@ -2665,8 +2695,11 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0724688A-8298-4485-ACBD-A429C8451820}">
-  <dimension ref="A3:A14"/>
+  <dimension ref="A3:B27"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="37.26953125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="3" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
@@ -2708,6 +2741,54 @@
         <v>101</v>
       </c>
     </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>167</v>
+      </c>
+      <c r="B19" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A26" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A27" t="s">
+        <v>175</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>